<commit_message>
Fix AI path following hang when handleMove rejects a step
Two bugs fixed:
1. aiFollowPath: if handleMove rejects a move (MP insufficient, stacking,
   etc.), startDefensiveFire is never called, so afterDefensiveFire never
   fires and the entire callback chain breaks. All subsequent units stop
   processing. Fixed by detecting unmoved unit after handleMove and calling
   callback directly.

2. BFS backward penalty mismatch: BFS skipped backward penalty for
   justEntered units (!isFirst check) but handleMove always applies it.
   This caused BFS to underestimate cost by 1 MP, leading to handleMove
   rejecting valid BFS paths.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tanks+/シナリオ.xlsx
+++ b/tanks+/シナリオ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baron/Desktop/aigame/tanks+/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F417A7-C447-974E-8232-AA3B014BD3A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A2FF82-585A-6D4A-B1CB-92CC64C6EB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="24980" windowHeight="16480" xr2:uid="{7F6B04F6-64B6-744D-8C71-D51E5E1F5DF2}"/>
+    <workbookView xWindow="5220" yWindow="660" windowWidth="20980" windowHeight="16440" xr2:uid="{7F6B04F6-64B6-744D-8C71-D51E5E1F5DF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="68">
   <si>
     <t>赤軍の反抗</t>
     <rPh sb="0" eb="2">
@@ -410,6 +410,114 @@
       <t xml:space="preserve">ハカイ </t>
     </rPh>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>カーン近郊</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>歩兵</t>
+    <rPh sb="0" eb="2">
+      <t xml:space="preserve">ホヘイ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>tiger1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>クロムウエル</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ファイアフライ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>あり</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ⅴ号駆逐戦車</t>
+    <rPh sb="1" eb="2">
+      <t xml:space="preserve">ゴウ </t>
+    </rPh>
+    <rPh sb="2" eb="6">
+      <t xml:space="preserve">クチクセンシャ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>マーダーⅢ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ⅲ号突撃</t>
+    <rPh sb="1" eb="2">
+      <t xml:space="preserve">ゴウ </t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t xml:space="preserve">トツゲキ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>建物を支配している</t>
+    <rPh sb="0" eb="2">
+      <t xml:space="preserve">タテモノヲシハイシテイル </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>map-C</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>右から侵入</t>
+    <rPh sb="0" eb="1">
+      <t xml:space="preserve">ミギ </t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t xml:space="preserve">シンニュウ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>左から侵入</t>
+    <rPh sb="0" eb="1">
+      <t xml:space="preserve">ヒダリ </t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t xml:space="preserve">シンニュウ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>5ターンに増援</t>
+    <rPh sb="5" eb="7">
+      <t xml:space="preserve">ゾウエン </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ダイス1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ダイス2</t>
+  </si>
+  <si>
+    <t>ダイス3</t>
+  </si>
+  <si>
+    <t>ダイス4</t>
+  </si>
+  <si>
+    <t>ダイス5</t>
+  </si>
+  <si>
+    <t>ダイス6</t>
   </si>
 </sst>
 </file>
@@ -771,17 +879,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1691EB29-040A-E845-93D2-743CE4AB08D0}">
-  <dimension ref="B2:N16"/>
+  <dimension ref="B2:P24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="23"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.25" customWidth="1"/>
-    <col min="12" max="12" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.75" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.25" customWidth="1"/>
+    <col min="13" max="13" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14">
+    <row r="2" spans="2:15">
       <c r="B2" t="s">
         <v>17</v>
       </c>
@@ -800,23 +908,23 @@
       <c r="H2" t="s">
         <v>5</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>26</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>27</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>13</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>20</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="2:14">
+    <row r="3" spans="2:15">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -838,23 +946,23 @@
       <c r="H3" t="s">
         <v>6</v>
       </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
       <c r="J3" t="s">
         <v>28</v>
       </c>
       <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" t="s">
         <v>14</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>15</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:14">
+    <row r="4" spans="2:15">
       <c r="C4" t="s">
         <v>9</v>
       </c>
@@ -868,7 +976,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:14">
+    <row r="5" spans="2:15">
       <c r="E5" t="s">
         <v>12</v>
       </c>
@@ -876,7 +984,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:14">
+    <row r="7" spans="2:15">
       <c r="B7" t="s">
         <v>18</v>
       </c>
@@ -892,23 +1000,23 @@
       <c r="H7" t="s">
         <v>6</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>24</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>25</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>14</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>22</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="2:14">
+    <row r="8" spans="2:15">
       <c r="C8" t="s">
         <v>19</v>
       </c>
@@ -922,7 +1030,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:14">
+    <row r="9" spans="2:15">
       <c r="E9" t="s">
         <v>11</v>
       </c>
@@ -930,7 +1038,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:14">
+    <row r="10" spans="2:15">
       <c r="E10" t="s">
         <v>12</v>
       </c>
@@ -938,7 +1046,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:14">
+    <row r="11" spans="2:15">
       <c r="B11" t="s">
         <v>40</v>
       </c>
@@ -954,23 +1062,23 @@
       <c r="H11" t="s">
         <v>6</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>47</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>25</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>45</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>46</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="2:14">
+    <row r="12" spans="2:15">
       <c r="C12" t="s">
         <v>41</v>
       </c>
@@ -984,7 +1092,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="2:14">
+    <row r="13" spans="2:15">
       <c r="C13" t="s">
         <v>9</v>
       </c>
@@ -998,7 +1106,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="2:14">
+    <row r="14" spans="2:15">
       <c r="C14" t="s">
         <v>42</v>
       </c>
@@ -1006,30 +1114,30 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="2:14">
+    <row r="15" spans="2:15">
       <c r="C15" t="s">
         <v>1</v>
       </c>
       <c r="E15" t="s">
         <v>35</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>1</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>35</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>20</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>32</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="2:14">
+    <row r="16" spans="2:15">
       <c r="B16" t="s">
         <v>29</v>
       </c>
@@ -1051,23 +1159,154 @@
       <c r="H16" t="s">
         <v>6</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>37</v>
       </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>36</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>14</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>33</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>34</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16">
+      <c r="B18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18">
+        <v>6</v>
+      </c>
+      <c r="G18">
+        <v>10</v>
+      </c>
+      <c r="H18" t="s">
+        <v>53</v>
+      </c>
+      <c r="J18" t="s">
+        <v>57</v>
+      </c>
+      <c r="K18" t="s">
+        <v>57</v>
+      </c>
+      <c r="L18" t="s">
+        <v>58</v>
+      </c>
+      <c r="M18" t="s">
+        <v>59</v>
+      </c>
+      <c r="N18" t="s">
+        <v>60</v>
+      </c>
+      <c r="O18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16">
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="H19" t="s">
+        <v>54</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+      <c r="O19" t="s">
+        <v>62</v>
+      </c>
+      <c r="P19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16">
+      <c r="C20" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="H20" t="s">
+        <v>9</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="O20" t="s">
+        <v>63</v>
+      </c>
+      <c r="P20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:16">
+      <c r="H21" t="s">
+        <v>55</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="O21" t="s">
+        <v>64</v>
+      </c>
+      <c r="P21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16">
+      <c r="H22" t="s">
+        <v>56</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="O22" t="s">
+        <v>65</v>
+      </c>
+      <c r="P22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="2:16">
+      <c r="O23" t="s">
+        <v>66</v>
+      </c>
+      <c r="P23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="2:16">
+      <c r="O24" t="s">
+        <v>67</v>
+      </c>
+      <c r="P24" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add eliminate button for no-retreat units and undo-move button
- Retreat panel: "退却先なし" text is now a clickable button that
  eliminates the unit and advances game state (fixes freeze when
  surrounded unit has DD result with no retreat hexes)
- Unit select panel: added "移動やり直し" button that reverts the
  last moved unit to its original hex (restores acted/movePath/mustAttack)
- Handles mech-pair stacking undo correctly
- Returns to select phase if currently in attack phase

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tanks+/シナリオ.xlsx
+++ b/tanks+/シナリオ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baron/Desktop/aigame/tanks+/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2573FCB-1299-0149-A258-3B160477710D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A65D9B7-3766-4248-98FA-1849C43C3171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3320" yWindow="660" windowWidth="22880" windowHeight="16440" xr2:uid="{7F6B04F6-64B6-744D-8C71-D51E5E1F5DF2}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="22880" windowHeight="16440" xr2:uid="{7F6B04F6-64B6-744D-8C71-D51E5E1F5DF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="80">
   <si>
     <t>赤軍の反抗</t>
     <rPh sb="0" eb="2">
@@ -280,26 +280,6 @@
   </si>
   <si>
     <t>アメリカスタート</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>下から侵入</t>
-    <rPh sb="0" eb="1">
-      <t xml:space="preserve">シタカラ </t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t xml:space="preserve">シンニュウ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>上から侵入</t>
-    <rPh sb="0" eb="1">
-      <t xml:space="preserve">ウエカラ </t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t xml:space="preserve">シンニュウ </t>
-    </rPh>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -1144,7 +1124,7 @@
     </row>
     <row r="11" spans="2:14">
       <c r="B11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
@@ -1156,22 +1136,22 @@
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L11" t="s">
         <v>14</v>
       </c>
       <c r="M11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="N11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="2:14">
@@ -1194,7 +1174,7 @@
         <v>2</v>
       </c>
       <c r="L12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="2:14">
@@ -1211,7 +1191,7 @@
         <v>15</v>
       </c>
       <c r="H13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -1227,7 +1207,7 @@
     </row>
     <row r="16" spans="2:14">
       <c r="B16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -1242,16 +1222,16 @@
         <v>6</v>
       </c>
       <c r="J16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K16" t="s">
         <v>25</v>
       </c>
       <c r="L16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="M16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N16" t="s">
         <v>23</v>
@@ -1259,13 +1239,13 @@
     </row>
     <row r="17" spans="2:16">
       <c r="C17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D17">
         <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F17">
         <v>5</v>
@@ -1279,7 +1259,7 @@
         <v>2</v>
       </c>
       <c r="E18" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F18">
         <v>10</v>
@@ -1287,7 +1267,7 @@
     </row>
     <row r="19" spans="2:16">
       <c r="C19" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D19">
         <v>3</v>
@@ -1295,7 +1275,7 @@
     </row>
     <row r="21" spans="2:16">
       <c r="B21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C21" t="s">
         <v>1</v>
@@ -1310,30 +1290,30 @@
         <v>6</v>
       </c>
       <c r="J21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L21" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="M21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="N21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="2:16">
       <c r="C22" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D22">
         <v>4</v>
       </c>
       <c r="E22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F22">
         <v>8</v>
@@ -1350,7 +1330,7 @@
         <v>2</v>
       </c>
       <c r="E23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F23">
         <v>10</v>
@@ -1358,13 +1338,13 @@
     </row>
     <row r="24" spans="2:16">
       <c r="C24" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D24">
         <v>4</v>
       </c>
       <c r="E24" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F24">
         <v>2</v>
@@ -1375,13 +1355,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J26" t="s">
         <v>1</v>
       </c>
       <c r="K26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M26" t="s">
         <v>20</v>
@@ -1390,7 +1370,7 @@
         <v>32</v>
       </c>
       <c r="O26" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="2:16">
@@ -1416,36 +1396,36 @@
         <v>6</v>
       </c>
       <c r="J27" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K27" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L27" t="s">
         <v>14</v>
       </c>
       <c r="M27" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="N27" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="O27" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="B29" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D29">
         <v>2</v>
       </c>
       <c r="E29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F29">
         <v>6</v>
@@ -1454,51 +1434,51 @@
         <v>10</v>
       </c>
       <c r="H29" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J29" t="s">
+        <v>55</v>
+      </c>
+      <c r="K29" t="s">
+        <v>55</v>
+      </c>
+      <c r="L29" t="s">
+        <v>56</v>
+      </c>
+      <c r="M29" t="s">
         <v>57</v>
       </c>
-      <c r="K29" t="s">
-        <v>57</v>
-      </c>
-      <c r="L29" t="s">
+      <c r="N29" t="s">
         <v>58</v>
       </c>
-      <c r="M29" t="s">
+      <c r="O29" t="s">
         <v>59</v>
-      </c>
-      <c r="N29" t="s">
-        <v>60</v>
-      </c>
-      <c r="O29" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="30" spans="2:16">
       <c r="C30" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D30">
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F30">
         <v>2</v>
       </c>
       <c r="H30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I30">
         <v>1</v>
       </c>
       <c r="O30" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="P30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="2:16">
@@ -1515,7 +1495,7 @@
         <v>1</v>
       </c>
       <c r="O31" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="P31" t="s">
         <v>9</v>
@@ -1523,52 +1503,52 @@
     </row>
     <row r="32" spans="2:16">
       <c r="H32" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I32">
         <v>1</v>
       </c>
       <c r="O32" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P32" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="2:16">
       <c r="H33" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I33">
         <v>1</v>
       </c>
       <c r="O33" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="P33" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="2:16">
       <c r="O34" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P34" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="2:16">
       <c r="B35" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D35">
         <v>2</v>
       </c>
       <c r="E35" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F35">
         <v>4</v>
@@ -1580,10 +1560,10 @@
         <v>6</v>
       </c>
       <c r="J35" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="K35" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L35" t="s">
         <v>14</v>
@@ -1591,19 +1571,19 @@
     </row>
     <row r="36" spans="2:16">
       <c r="C36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D36">
         <v>2</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F36">
         <v>4</v>
       </c>
       <c r="L36" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="2:16">
@@ -1614,7 +1594,7 @@
         <v>4</v>
       </c>
       <c r="E37" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F37">
         <v>4</v>

</xml_diff>